<commit_message>
refactor: ♻️ Unifica benchmark em um script (verifica + mede + planilha)
Adiciona scripts/benchmark.py com as 3 fases (verificacao de entrada/saida,
medicao de tempos e geracao do xlsx) e remove os scripts que ele substitui
(executa_benchmark, verifica_benchmark, planilha_benchmark).
</commit_message>
<xml_diff>
--- a/arquivos/xlsx/tempos_execucao.xlsx
+++ b/arquivos/xlsx/tempos_execucao.xlsx
@@ -620,79 +620,79 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>13.1</v>
+        <v>12.7885</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>13.2859</v>
+        <v>12.703</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.3106</v>
+        <v>1.3347</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.2096</v>
+        <v>0.2107</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>5.2916</v>
+        <v>5.1228</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0.0021</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>4.7541</v>
+        <v>4.8346</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>51.3047</v>
+        <v>51.4528</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>2.0911</v>
+        <v>2.099</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.452</v>
+        <v>0.4531</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.8354</v>
+        <v>0.4887</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>1.3045</v>
+        <v>1.3321</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>66.3489</v>
+        <v>66.2766</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.0258</v>
+        <v>0.0256</v>
       </c>
       <c r="P2" s="3" t="n">
         <v>0.0012</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.6666</v>
+        <v>0.6624</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>0.1125</v>
+        <v>0.1122</v>
       </c>
       <c r="T2" s="3" t="n">
-        <v>0.0106</v>
+        <v>0.0144</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>1.2787</v>
+        <v>1.1599</v>
       </c>
       <c r="V2" s="3" t="n">
-        <v>4.4557</v>
+        <v>4.4406</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>0.0051</v>
+        <v>0.005</v>
       </c>
       <c r="X2" s="3" t="n">
-        <v>0.1539</v>
+        <v>0.1594</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>0.1422</v>
+        <v>0.1406</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>1.9323</v>
+        <v>1.8885</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -702,16 +702,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>8.2751</v>
+        <v>8.299899999999999</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>5.5398</v>
+        <v>5.4972</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.5004999999999999</v>
+        <v>0.5052</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.1204</v>
+        <v>0.1198</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -729,13 +729,13 @@
         </is>
       </c>
       <c r="I3" s="5" t="n">
-        <v>9.170299999999999</v>
+        <v>8.9918</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>1.0499</v>
+        <v>1.0216</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.4</v>
+        <v>0.399</v>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="P3" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.001</v>
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="R3" s="5" t="n">
-        <v>0.638</v>
+        <v>0.6384</v>
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
@@ -794,13 +794,13 @@
         </is>
       </c>
       <c r="X3" s="5" t="n">
-        <v>0.1914</v>
+        <v>0.1553</v>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>0.0755</v>
+        <v>0.075</v>
       </c>
       <c r="Z3" s="5" t="n">
-        <v>0.8843</v>
+        <v>0.8852</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
@@ -809,80 +809,82 @@
           <t>Tempo_Iteracao_Media</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>21.3974</v>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>14.5799</v>
+        <v>14.1194</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3.7735</v>
+        <v>3.8713</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.5591</v>
+        <v>0.7418</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5.3046</v>
+        <v>5.1612</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.0133</v>
+        <v>0.013</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>18.8517</v>
+        <v>18.8274</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>55.2038</v>
+        <v>55.5665</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>2.6453</v>
+        <v>2.5537</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.8139</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>1.4972</v>
+        <v>1.164</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>2.137</v>
+        <v>2.074</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>475.0938</v>
+        <v>469.5075</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.0346</v>
+        <v>0.0344</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.0068</v>
+        <v>0.0073</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.0288</v>
+        <v>0.0275</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.8054</v>
+        <v>0.8141</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.9122</v>
+        <v>0.9066</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>15155.1277</v>
+        <v>15118.6413</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>1.4763</v>
+        <v>1.4987</v>
       </c>
       <c r="V4" s="3" t="n">
-        <v>2.726</v>
+        <v>2.7205</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>0.0171</v>
+        <v>0.0172</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>0.2647</v>
+        <v>0.265</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>0.5054999999999999</v>
+        <v>0.4974</v>
       </c>
       <c r="Z4" s="3" t="n">
-        <v>2.2489</v>
+        <v>2.2492</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">

</xml_diff>

<commit_message>
refactor: ♻️ Torna a duração piso do modo por tempo e reporta métricas exatas
O ramo por tempo do driver agora itera lotes de iterações completas até a
soma dos tempos alcançar >= T (antes, um lote único estimado podia parar
aquém do alvo) e reporta iterações exatas, tempo total e ms por chamada,
eliminando o float normalizado. Atualiza o runner (--duracao: novo regex e
CSV com piso_s/iteracoes/tempo_total_s/tempo_ms_por_chamada), as docs e os
resultados regenerados (csv/xlsx).
</commit_message>
<xml_diff>
--- a/arquivos/xlsx/tempos_execucao.xlsx
+++ b/arquivos/xlsx/tempos_execucao.xlsx
@@ -489,127 +489,127 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Fibonaccil(500.000)</t>
+          <t>Fibonacci</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Factorial(50.000, 1)</t>
+          <t>Factorial</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Sum (5.000.000)</t>
+          <t>Sum</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>mdc(fib(500), fib(501))</t>
+          <t>mdc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>woodcutter([1, ..., 100001), 1250025000, 0, max(arvores))</t>
+          <t>woodcutter</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Binary_Search_Tree()</t>
+          <t>Binary_Search_Tree</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>quick_select()</t>
+          <t>quick_select</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>identical_strings()</t>
+          <t>identical_strings</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>linear_search()</t>
+          <t>linear_search</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>non_negative_int_contain_digit()</t>
+          <t>non_negative_int_contain_digit</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Hannoi (20)</t>
+          <t>Hannoi</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>MergeSort(1.000.000)</t>
+          <t>MergeSort</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>NumSearchTree (18)</t>
+          <t>NumSearchTree</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>fast_pow(2, 10.000)</t>
+          <t>fast_pow</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>count_bits((1 &lt;&lt; 20) - 1)</t>
+          <t>count_bits</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>flatten()</t>
+          <t>flatten</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>first_missing(range(500))</t>
+          <t>first_missing</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>is_valid_bst(1.000)</t>
+          <t>is_valid_bst</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>fib_memo(35)</t>
+          <t>fib_memo</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>countdown(500)</t>
+          <t>countdown</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>safe_parse(['1','abc','3',None,'5'] * 200)</t>
+          <t>safe_parse</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>sum_nested()</t>
+          <t>sum_nested</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>remove_keys(dict)</t>
+          <t>remove_keys</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>find_first(range(1.000), x &gt; 5000)</t>
+          <t>find_first</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>count_matches([1,2,3] * 333, 2)</t>
+          <t>count_matches</t>
         </is>
       </c>
     </row>
@@ -620,79 +620,79 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>12.7885</v>
+        <v>14.8534</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>12.703</v>
+        <v>13.8094</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.3347</v>
+        <v>1.4476</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.2107</v>
+        <v>0.2047</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>5.1228</v>
+        <v>5.1315</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0.0021</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>4.8346</v>
+        <v>4.8613</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>51.4528</v>
+        <v>53.4375</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>2.099</v>
+        <v>2.1149</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.4531</v>
+        <v>0.452</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.4887</v>
+        <v>0.5016</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>1.3321</v>
+        <v>1.3144</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>66.2766</v>
+        <v>65.8858</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.0256</v>
+        <v>0.026</v>
       </c>
       <c r="P2" s="3" t="n">
         <v>0.0012</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.6624</v>
+        <v>0.6776</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>0.1122</v>
+        <v>0.1189</v>
       </c>
       <c r="T2" s="3" t="n">
-        <v>0.0144</v>
+        <v>0.0098</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>1.1599</v>
+        <v>1.2886</v>
       </c>
       <c r="V2" s="3" t="n">
-        <v>4.4406</v>
+        <v>4.5549</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>0.005</v>
+        <v>0.0048</v>
       </c>
       <c r="X2" s="3" t="n">
-        <v>0.1594</v>
+        <v>0.1609</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>0.1406</v>
+        <v>0.1456</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>1.8885</v>
+        <v>1.9991</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -702,16 +702,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>8.299899999999999</v>
+        <v>8.103899999999999</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>5.4972</v>
+        <v>5.5101</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.5052</v>
+        <v>0.5244</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.1198</v>
+        <v>0.1789</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -729,13 +729,13 @@
         </is>
       </c>
       <c r="I3" s="5" t="n">
-        <v>8.9918</v>
+        <v>9.1958</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>1.0216</v>
+        <v>1.039</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.399</v>
+        <v>0.4007</v>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="P3" s="5" t="n">
-        <v>0.001</v>
+        <v>0.0009</v>
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="R3" s="5" t="n">
-        <v>0.6384</v>
+        <v>0.6389</v>
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
@@ -794,13 +794,13 @@
         </is>
       </c>
       <c r="X3" s="5" t="n">
-        <v>0.1553</v>
+        <v>0.16</v>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>0.075</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="Z3" s="5" t="n">
-        <v>0.8852</v>
+        <v>0.903</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
@@ -809,82 +809,80 @@
           <t>Tempo_Iteracao_Media</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B4" s="3" t="n">
+        <v>22.0758</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>14.1194</v>
+        <v>15.5909</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3.8713</v>
+        <v>3.9393</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.7418</v>
+        <v>0.6764</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5.1612</v>
+        <v>5.3159</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0.013</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>18.8274</v>
+        <v>19.1035</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>55.5665</v>
+        <v>57.6152</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>2.5537</v>
+        <v>2.6075</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.8114</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>1.164</v>
+        <v>1.1746</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>2.074</v>
+        <v>2.0728</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>469.5075</v>
+        <v>472.0944</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.0344</v>
+        <v>0.0349</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.0073</v>
+        <v>0.0072</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.0283</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.8141</v>
+        <v>0.8051</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.9066</v>
+        <v>0.9238</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>15118.6413</v>
+        <v>15063.2199</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>1.4987</v>
+        <v>1.4943</v>
       </c>
       <c r="V4" s="3" t="n">
-        <v>2.7205</v>
+        <v>2.7216</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>0.0172</v>
+        <v>0.017</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>0.265</v>
+        <v>0.272</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>0.4974</v>
+        <v>0.4861</v>
       </c>
       <c r="Z4" s="3" t="n">
-        <v>2.2492</v>
+        <v>2.3231</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">

</xml_diff>